<commit_message>
Donna meeting sheet: add WhatsApp Business API tab
</commit_message>
<xml_diff>
--- a/niumee/Donna_Meeting_03Aug.xlsx
+++ b/niumee/Donna_Meeting_03Aug.xlsx
@@ -10,6 +10,7 @@
     <sheet name="1 Answer these" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="2 Tell her" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="3 Decisions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="4 WhatsApp Business API" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,6 +66,12 @@
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="7">
@@ -126,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -160,6 +167,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1219,4 +1230,221 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="66" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="13" t="inlineStr">
+        <is>
+          <t>Moving Nima to the official WhatsApp Business API</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Niumee already has a verified number, so the slow part (Meta business verification) is done. What is left is collecting five details from whoever administers it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>What we need</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Where it comes from / why</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="62" customHeight="1">
+      <c r="A5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>FIRST: is the number managed directly by Niumee in Meta Business Manager, or through a provider such as Twilio, 360dialog, Vonage or Infobip?</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>This decides everything. Managed directly means we can connect in a day. Held by a provider means the number is locked to them and has to be migrated out first, which needs their release and takes longer. Ask this one before anything else.</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6" ht="62" customHeight="1">
+      <c r="A6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Who is an ADMIN on the Meta Business account?</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>We need an admin to create a system user and issue a token. Usually IT or marketing, not reception.</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7" ht="62" customHeight="1">
+      <c r="A7" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>WhatsApp Business Account ID (WABA ID)</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Meta Business Manager, WhatsApp Accounts. It is a long number, not a name.</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8" ht="62" customHeight="1">
+      <c r="A8" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Phone Number ID</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Inside the WABA, under phone numbers. This is NOT the phone number itself, it is a separate numeric id. Both are needed.</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9" ht="62" customHeight="1">
+      <c r="A9" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>A permanent access token</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Created from a System User with the whatsapp_business_messaging and whatsapp_business_management permissions. Temporary tokens expire in 24 hours and would take Nima down again, so it must be the permanent kind.</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10" ht="62" customHeight="1">
+      <c r="A10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Which number will clients write to?</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>35699719066 is already set up on our side but clients do not know it. 35679002386 is the number clients actually use, but it must first be removed from normal WhatsApp, and reception would lose that chat on the handset. This is a commercial decision, not a technical one.</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11" ht="62" customHeight="1">
+      <c r="A11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Is the verified number already sending on another system?</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>A number can only belong to one WhatsApp Business account at a time. If marketing already uses it for campaigns, we need to know before touching it.</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>What changes for Nima</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>- Nobody can disconnect it by unlinking a device. Friday's outage becomes impossible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>- Outside 24 hours of a client's last message, only pre-approved templates may be sent. Inside 24 hours, anything.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>- Nima only ever replies, so day to day nothing changes for her.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>- Appointment reminders would become templates that Meta AND Donna approve before any go out. After the 31 July incident that is a control worth having.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>- Everything already built stays as it is. Only the connection underneath changes.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Donna sheet: Nima number is dedicated, migrate 35679002386
</commit_message>
<xml_diff>
--- a/niumee/Donna_Meeting_03Aug.xlsx
+++ b/niumee/Donna_Meeting_03Aug.xlsx
@@ -1238,7 +1238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1364,17 +1364,17 @@
       <c r="D9" s="6" t="inlineStr"/>
     </row>
     <row r="10" ht="62" customHeight="1">
-      <c r="A10" s="4" t="n">
+      <c r="A10" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Which number will clients write to?</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>35699719066 is already set up on our side but clients do not know it. 35679002386 is the number clients actually use, but it must first be removed from normal WhatsApp, and reception would lose that chat on the handset. This is a commercial decision, not a technical one.</t>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Is 35679002386 the number that is already verified, or is the verified one different?</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>35679002386 is Nima's dedicated line and reception has their own, so keeping it is the obvious choice: clients already write to it and nobody loses a chat. We just need to know whether it is already in the Meta account or has to be added to it.</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr"/>
@@ -1385,53 +1385,69 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Is the verified number already sending on another system?</t>
+          <t>Confirm we may delete 35679002386 from normal WhatsApp</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>A number can only belong to one WhatsApp Business account at a time. If marketing already uses it for campaigns, we need to know before touching it.</t>
+          <t>A number cannot be on the Cloud API and on the normal WhatsApp app at the same time. It has to be removed from the app first. Because it is Nima's line only, nothing operational is lost, and every client conversation is already stored on our side. It is a one way step, so we want it said out loud.</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr"/>
     </row>
-    <row r="13">
-      <c r="B13" s="15" t="inlineStr">
+    <row r="12" ht="62" customHeight="1">
+      <c r="A12" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Is 35679002386 already sending from another system?</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>A number can only belong to one WhatsApp Business account at a time. If marketing ever used it for campaigns we need to know before touching it.</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>What changes for Nima</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="16" t="inlineStr">
-        <is>
-          <t>- Nobody can disconnect it by unlinking a device. Friday's outage becomes impossible.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="16" t="inlineStr">
         <is>
-          <t>- Outside 24 hours of a client's last message, only pre-approved templates may be sent. Inside 24 hours, anything.</t>
+          <t>- Nobody can disconnect it by unlinking a device. Friday's outage becomes impossible.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="16" t="inlineStr">
         <is>
-          <t>- Nima only ever replies, so day to day nothing changes for her.</t>
+          <t>- Outside 24 hours of a client's last message, only pre-approved templates may be sent. Inside 24 hours, anything.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="16" t="inlineStr">
         <is>
-          <t>- Appointment reminders would become templates that Meta AND Donna approve before any go out. After the 31 July incident that is a control worth having.</t>
+          <t>- Nima only ever replies, so day to day nothing changes for her.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>- Appointment reminders would become templates that Meta AND Donna approve before any go out. After the 31 July incident that is a control worth having.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="16" t="inlineStr">
         <is>
           <t>- Everything already built stays as it is. Only the connection underneath changes.</t>
         </is>
@@ -1441,7 +1457,7 @@
   <mergeCells count="5">
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B19:C19"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="B18:C18"/>
   </mergeCells>

</xml_diff>